<commit_message>
Update S6 Group A: add Nagham Alqaq (5th member, QA/Software Tester)
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/birzeit/comp433/Project_section_6/COMP433_Section6_Allocations.xlsx
+++ b/birzeit/comp433/Project_section_6/COMP433_Section6_Allocations.xlsx
@@ -131,7 +131,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -153,11 +153,88 @@
         <color rgb="00BFC8D1"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFC8D1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFC8D1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFC8D1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFC8D1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFC8D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFC8D1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFC8D1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFC8D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFC8D1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFC8D1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFC8D1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFC8D1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFC8D1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BFC8D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -279,6 +356,9 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -689,6 +769,9 @@
           <t>7 groups</t>
         </is>
       </c>
+      <c r="D5" s="41" t="n"/>
+      <c r="E5" s="41" t="n"/>
+      <c r="F5" s="42" t="n"/>
     </row>
     <row r="6" ht="19" customHeight="1">
       <c r="A6" s="4" t="inlineStr"/>
@@ -702,6 +785,9 @@
           <t>1 group</t>
         </is>
       </c>
+      <c r="D6" s="41" t="n"/>
+      <c r="E6" s="41" t="n"/>
+      <c r="F6" s="42" t="n"/>
     </row>
     <row r="7" ht="19" customHeight="1">
       <c r="A7" s="6" t="inlineStr"/>
@@ -715,6 +801,9 @@
           <t>2 groups</t>
         </is>
       </c>
+      <c r="D7" s="41" t="n"/>
+      <c r="E7" s="41" t="n"/>
+      <c r="F7" s="42" t="n"/>
     </row>
     <row r="8" ht="19" customHeight="1">
       <c r="A8" s="8" t="inlineStr"/>
@@ -728,6 +817,9 @@
           <t>1 group (Group C — see note)</t>
         </is>
       </c>
+      <c r="D8" s="41" t="n"/>
+      <c r="E8" s="41" t="n"/>
+      <c r="F8" s="42" t="n"/>
     </row>
     <row r="9" ht="19" customHeight="1">
       <c r="A9" s="10" t="inlineStr"/>
@@ -741,6 +833,9 @@
           <t>1 group (Group J)</t>
         </is>
       </c>
+      <c r="D9" s="41" t="n"/>
+      <c r="E9" s="41" t="n"/>
+      <c r="F9" s="42" t="n"/>
     </row>
     <row r="10" ht="19" customHeight="1">
       <c r="A10" s="10" t="inlineStr"/>
@@ -754,6 +849,9 @@
           <t>64 — Vaccination drive coordination</t>
         </is>
       </c>
+      <c r="D10" s="41" t="n"/>
+      <c r="E10" s="41" t="n"/>
+      <c r="F10" s="42" t="n"/>
     </row>
     <row r="11" ht="6" customHeight="1"/>
     <row r="12" ht="24" customHeight="1">
@@ -823,7 +921,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>4 members: Mohammed Jadaa, Ahmad Masri, Yanal Omar, Saja Sayara</t>
+          <t>5 members: Nagham Alqaq, Mohammed Jadaa, Ahmad Masri, Yanal Omar, Saja Sayara</t>
         </is>
       </c>
     </row>
@@ -1617,13 +1715,23 @@
           <t>• Group F (originally K, single member: Adam Khabisa) was collapsed. Adam joined Group I (now Group H), which is now a 5-member team.</t>
         </is>
       </c>
+      <c r="B44" s="41" t="n"/>
+      <c r="C44" s="41" t="n"/>
+      <c r="D44" s="41" t="n"/>
+      <c r="E44" s="41" t="n"/>
+      <c r="F44" s="42" t="n"/>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="22" t="inlineStr">
         <is>
-          <t>• Intisar Assi moved from Group A to Group L (originally Z) by her email request. Group L is now a 5-member all-female team. Group A drops to 4 members, which is still valid.</t>
-        </is>
-      </c>
+          <t>• Intisar Assi was not in any group in the Phase 0 preferences file. She was added to Group L (originally Z) as a fifth member by her request. Nagham Alqaq was incorrectly omitted from Group A in the initial workbook build; she has been restored. Group A has 5 members; Group L has 5 members.</t>
+        </is>
+      </c>
+      <c r="B45" s="41" t="n"/>
+      <c r="C45" s="41" t="n"/>
+      <c r="D45" s="41" t="n"/>
+      <c r="E45" s="41" t="n"/>
+      <c r="F45" s="42" t="n"/>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="22" t="inlineStr">
@@ -1631,6 +1739,11 @@
           <t>• Group C did not receive any of its top three preferences. All three (54, 55, 61) were the first choice of three other groups (B, J, H respectively); the Hungarian assignment minimised total disappointment by placing C on business 56 (Lab test booking and results), which is closest in spirit to its top picks (clinical/service domains).</t>
         </is>
       </c>
+      <c r="B46" s="41" t="n"/>
+      <c r="C46" s="41" t="n"/>
+      <c r="D46" s="41" t="n"/>
+      <c r="E46" s="41" t="n"/>
+      <c r="F46" s="42" t="n"/>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="22" t="inlineStr">
@@ -1638,6 +1751,11 @@
           <t>• Group J (originally T) submitted no preferences. They have been allocated business 58 (Physiotherapy clinic) from the unassigned pool. They must confirm their management strategy and roles before Phase 1 begins.</t>
         </is>
       </c>
+      <c r="B47" s="41" t="n"/>
+      <c r="C47" s="41" t="n"/>
+      <c r="D47" s="41" t="n"/>
+      <c r="E47" s="41" t="n"/>
+      <c r="F47" s="42" t="n"/>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="22" t="inlineStr">
@@ -1645,6 +1763,11 @@
           <t>• Group K (originally Y) submitted partial management strategy ("4, 2"); we have interpreted this as "online + voting" with weekly cadence as the default. They should confirm.</t>
         </is>
       </c>
+      <c r="B48" s="41" t="n"/>
+      <c r="C48" s="41" t="n"/>
+      <c r="D48" s="41" t="n"/>
+      <c r="E48" s="41" t="n"/>
+      <c r="F48" s="42" t="n"/>
     </row>
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="22" t="inlineStr">
@@ -1652,6 +1775,11 @@
           <t>• Business 64 (Vaccination drive coordination) is unallocated and held as a buffer in case any group needs to switch.</t>
         </is>
       </c>
+      <c r="B49" s="41" t="n"/>
+      <c r="C49" s="41" t="n"/>
+      <c r="D49" s="41" t="n"/>
+      <c r="E49" s="41" t="n"/>
+      <c r="F49" s="42" t="n"/>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="22" t="inlineStr">
@@ -1659,6 +1787,11 @@
           <t>• The cycle has 12 groups: A → B → C → D → E → F → G → H → I → J → K → L → A.</t>
         </is>
       </c>
+      <c r="B50" s="41" t="n"/>
+      <c r="C50" s="41" t="n"/>
+      <c r="D50" s="41" t="n"/>
+      <c r="E50" s="41" t="n"/>
+      <c r="F50" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="19">
@@ -1766,26 +1899,36 @@
           <t>Member 1</t>
         </is>
       </c>
+      <c r="G4" s="41" t="n"/>
+      <c r="H4" s="42" t="n"/>
       <c r="I4" s="12" t="inlineStr">
         <is>
           <t>Member 2</t>
         </is>
       </c>
+      <c r="J4" s="41" t="n"/>
+      <c r="K4" s="42" t="n"/>
       <c r="L4" s="12" t="inlineStr">
         <is>
           <t>Member 3</t>
         </is>
       </c>
+      <c r="M4" s="41" t="n"/>
+      <c r="N4" s="42" t="n"/>
       <c r="O4" s="12" t="inlineStr">
         <is>
           <t>Member 4</t>
         </is>
       </c>
+      <c r="P4" s="41" t="n"/>
+      <c r="Q4" s="42" t="n"/>
       <c r="R4" s="12" t="inlineStr">
         <is>
           <t>Member 5</t>
         </is>
       </c>
+      <c r="S4" s="41" t="n"/>
+      <c r="T4" s="42" t="n"/>
       <c r="U4" s="12" t="inlineStr">
         <is>
           <t>Management strategy</t>
@@ -1798,6 +1941,11 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="43" t="n"/>
+      <c r="B5" s="43" t="n"/>
+      <c r="C5" s="43" t="n"/>
+      <c r="D5" s="43" t="n"/>
+      <c r="E5" s="43" t="n"/>
       <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Name</t>
@@ -1873,6 +2021,8 @@
           <t>Role(s)</t>
         </is>
       </c>
+      <c r="U5" s="43" t="n"/>
+      <c r="V5" s="43" t="n"/>
     </row>
     <row r="6" ht="50" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
@@ -1962,17 +2112,17 @@
       </c>
       <c r="R6" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Nagham Alqaq</t>
         </is>
       </c>
       <c r="S6" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1201970</t>
         </is>
       </c>
       <c r="T6" s="27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>QA / Software Tester</t>
         </is>
       </c>
       <c r="U6" s="4" t="inlineStr">
@@ -1982,7 +2132,7 @@
       </c>
       <c r="V6" s="14" t="inlineStr">
         <is>
-          <t>Intisar moved to Group L by request</t>
+          <t>Nagham Alqaq restored (was incorrectly omitted). Intisar Assi is in Group L.</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3324,7 @@
       </c>
       <c r="V17" s="20" t="inlineStr">
         <is>
-          <t>Intisar Assi joined from Group A by request</t>
+          <t>Intisar Assi joined Group L by her request (was unassigned in Phase 0 preferences).</t>
         </is>
       </c>
     </row>
@@ -3798,6 +3948,9 @@
           <t>Marking convention: phases are graded A / B / C / D, then converted to marks. Important: AI-generated UML diagrams are not allowed at any stage. Submitting AI-generated work will receive zero and may be referred to a disciplinary committee.</t>
         </is>
       </c>
+      <c r="B14" s="41" t="n"/>
+      <c r="C14" s="41" t="n"/>
+      <c r="D14" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>